<commit_message>
exel inclusion in public folder
</commit_message>
<xml_diff>
--- a/public/employees.xlsx
+++ b/public/employees.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
   <si>
     <t>gender</t>
   </si>
@@ -57,12 +57,6 @@
   </si>
   <si>
     <t>Date Of Hire</t>
-  </si>
-  <si>
-    <t>Date Of Termination</t>
-  </si>
-  <si>
-    <t>Profile Picture</t>
   </si>
   <si>
     <t>Salary</t>
@@ -404,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:N2"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="13.81640625" customWidth="1"/>
@@ -418,11 +412,10 @@
     <col min="9" max="9" width="14.1796875" customWidth="1"/>
     <col min="10" max="10" width="14.90625" customWidth="1"/>
     <col min="11" max="11" width="13.453125" customWidth="1"/>
-    <col min="12" max="12" width="23" customWidth="1"/>
-    <col min="13" max="13" width="17" customWidth="1"/>
+    <col min="12" max="12" width="15.6328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>7</v>
       </c>
@@ -459,16 +452,10 @@
       <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
-        <v>12</v>
-      </c>
-      <c r="N1" t="s">
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
         <v>13</v>
-      </c>
-    </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>15</v>
       </c>
       <c r="B2">
         <v>0</v>
@@ -480,7 +467,7 @@
         <v>62798098789</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="F2">
         <v>98778640997898</v>
@@ -489,7 +476,7 @@
         <v>0</v>
       </c>
       <c r="H2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="I2">
         <v>7867987</v>
@@ -499,6 +486,9 @@
       </c>
       <c r="K2" s="2">
         <v>44097</v>
+      </c>
+      <c r="L2">
+        <v>90000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>